<commit_message>
red mark zero information
</commit_message>
<xml_diff>
--- a/Data/xlxs/smartwatch_cleaned_statistics_fixed.xlsx
+++ b/Data/xlxs/smartwatch_cleaned_statistics_fixed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Smart-Watch-Stats-Project\Data\xlxs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{961A599E-31B7-4E1F-8A55-27919202F55C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2006AF5-59D5-4E3E-A4CA-B5C16CCD9FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Statistics" sheetId="1" r:id="rId1"/>
@@ -519,7 +519,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -529,6 +529,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF6161"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -545,80 +551,29 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="4" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="53">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="4" formatCode="#,##0.00"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Carlito"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -997,8 +952,67 @@
     <dxf>
       <numFmt numFmtId="4" formatCode="#,##0.00"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="4" formatCode="#,##0.00"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF6161"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1011,7 +1025,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{608EBCD2-6D24-4D23-891F-9723046FD8E9}" name="Table1" displayName="Table1" ref="B4:X35" totalsRowShown="0" headerRowDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{608EBCD2-6D24-4D23-891F-9723046FD8E9}" name="Table1" displayName="Table1" ref="B4:X35" totalsRowShown="0" headerRowDxfId="49">
   <autoFilter ref="B4:X35" xr:uid="{608EBCD2-6D24-4D23-891F-9723046FD8E9}"/>
   <tableColumns count="23">
     <tableColumn id="1" xr3:uid="{67458E5E-E663-4533-8FC4-1D9546780BBC}" name="Group Type"/>
@@ -1020,207 +1034,207 @@
     <tableColumn id="4" xr3:uid="{6CD379F3-D2D6-4BD2-B64A-92F429F1E655}" name="Model"/>
     <tableColumn id="5" xr3:uid="{3C2EB0A8-0BAD-4378-89F0-5BDD9153042B}" name="Platform"/>
     <tableColumn id="6" xr3:uid="{6CE3D0B5-1BD4-48B8-B479-E6E34C13ABDB}" name="n"/>
-    <tableColumn id="7" xr3:uid="{B132AE66-45FF-404C-8FE1-225BFA1B609B}" name="Price Mean" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{D93DD236-57DE-4C10-9C84-D6BFBB0CF138}" name="Price Median" dataDxfId="51"/>
-    <tableColumn id="9" xr3:uid="{441B8F93-59E0-44CB-975D-F74259024454}" name="Price SD" dataDxfId="50"/>
-    <tableColumn id="10" xr3:uid="{B596794B-3611-4E3E-8C66-54408D9A271E}" name="Price CV (%)" dataDxfId="49">
+    <tableColumn id="7" xr3:uid="{B132AE66-45FF-404C-8FE1-225BFA1B609B}" name="Price Mean" dataDxfId="48"/>
+    <tableColumn id="8" xr3:uid="{D93DD236-57DE-4C10-9C84-D6BFBB0CF138}" name="Price Median" dataDxfId="47"/>
+    <tableColumn id="9" xr3:uid="{441B8F93-59E0-44CB-975D-F74259024454}" name="Price SD" dataDxfId="46"/>
+    <tableColumn id="10" xr3:uid="{B596794B-3611-4E3E-8C66-54408D9A271E}" name="Price CV (%)" dataDxfId="45">
       <calculatedColumnFormula>IF(OR(G5&lt;2,H5=0),"",J5/H5*100)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{921DAC6C-48BB-427A-BCA1-B2F7243D1D39}" name="Price Min" dataDxfId="48"/>
-    <tableColumn id="12" xr3:uid="{62608AB5-9B27-4290-8269-58077B61222B}" name="Price Q1" dataDxfId="47"/>
-    <tableColumn id="13" xr3:uid="{2F9FDB44-93F4-438D-8D00-00ED156DAD26}" name="Price Q3" dataDxfId="46"/>
-    <tableColumn id="14" xr3:uid="{5244D297-7371-414A-A1CC-DFA9E941ABE8}" name="Price Max" dataDxfId="45"/>
+    <tableColumn id="11" xr3:uid="{921DAC6C-48BB-427A-BCA1-B2F7243D1D39}" name="Price Min" dataDxfId="44"/>
+    <tableColumn id="12" xr3:uid="{62608AB5-9B27-4290-8269-58077B61222B}" name="Price Q1" dataDxfId="43"/>
+    <tableColumn id="13" xr3:uid="{2F9FDB44-93F4-438D-8D00-00ED156DAD26}" name="Price Q3" dataDxfId="42"/>
+    <tableColumn id="14" xr3:uid="{5244D297-7371-414A-A1CC-DFA9E941ABE8}" name="Price Max" dataDxfId="41"/>
     <tableColumn id="15" xr3:uid="{3762D7F6-B63A-460C-8353-ED41BCD0B4AA}" name="Rating n"/>
-    <tableColumn id="16" xr3:uid="{DB1AA01E-EA6E-4CB1-B45C-8515EB6EA389}" name="Rating Mean" dataDxfId="44"/>
-    <tableColumn id="17" xr3:uid="{0C4BB8AE-B734-4655-994E-6D3AD5A32FF6}" name="Rating Median" dataDxfId="43"/>
-    <tableColumn id="18" xr3:uid="{723CB2AA-8C24-4054-9C00-5288D705A4F7}" name="Rating SD" dataDxfId="42"/>
-    <tableColumn id="19" xr3:uid="{64A1CFDD-7A08-49D7-88C1-32B0F5C32D77}" name="Rating CV (%)" dataDxfId="41">
+    <tableColumn id="16" xr3:uid="{DB1AA01E-EA6E-4CB1-B45C-8515EB6EA389}" name="Rating Mean" dataDxfId="40"/>
+    <tableColumn id="17" xr3:uid="{0C4BB8AE-B734-4655-994E-6D3AD5A32FF6}" name="Rating Median" dataDxfId="39"/>
+    <tableColumn id="18" xr3:uid="{723CB2AA-8C24-4054-9C00-5288D705A4F7}" name="Rating SD" dataDxfId="38"/>
+    <tableColumn id="19" xr3:uid="{64A1CFDD-7A08-49D7-88C1-32B0F5C32D77}" name="Rating CV (%)" dataDxfId="37">
       <calculatedColumnFormula>IF(OR(P5&lt;2,Q5=0),"",S5/Q5*100)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="20" xr3:uid="{19D7E071-1F24-4354-8655-D9889530DBA4}" name="Rating Min" dataDxfId="40"/>
-    <tableColumn id="21" xr3:uid="{C5278980-1389-465D-8C80-305B1ADD8D6D}" name="Rating Q1" dataDxfId="39"/>
-    <tableColumn id="22" xr3:uid="{BACFD2F4-8FD5-490E-8D52-8D4B7EA7B9D4}" name="Rating Q3" dataDxfId="38"/>
-    <tableColumn id="23" xr3:uid="{2E494D6A-E1BF-4418-B7A2-2A52C4EDF368}" name="Rating Max" dataDxfId="37"/>
+    <tableColumn id="20" xr3:uid="{19D7E071-1F24-4354-8655-D9889530DBA4}" name="Rating Min" dataDxfId="36"/>
+    <tableColumn id="21" xr3:uid="{C5278980-1389-465D-8C80-305B1ADD8D6D}" name="Rating Q1" dataDxfId="35"/>
+    <tableColumn id="22" xr3:uid="{BACFD2F4-8FD5-490E-8D52-8D4B7EA7B9D4}" name="Rating Q3" dataDxfId="34"/>
+    <tableColumn id="23" xr3:uid="{2E494D6A-E1BF-4418-B7A2-2A52C4EDF368}" name="Rating Max" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium5" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F2DFCB97-D8F8-46BD-9201-82BFE252AFB8}" name="Table10" displayName="Table10" ref="B2:G40" totalsRowShown="0" headerRowDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{F2DFCB97-D8F8-46BD-9201-82BFE252AFB8}" name="Table10" displayName="Table10" ref="B2:G40" totalsRowShown="0" headerRowDxfId="11">
   <autoFilter ref="B2:G40" xr:uid="{F2DFCB97-D8F8-46BD-9201-82BFE252AFB8}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{E40D0A5C-6A8E-4EEC-969B-40176608B52E}" name="brand"/>
     <tableColumn id="2" xr3:uid="{10E2567F-55BA-485A-BA52-B29BE75DD946}" name="model"/>
     <tableColumn id="3" xr3:uid="{3D2449CB-8CD3-42DA-8BDC-9148F035C97C}" name="platform"/>
     <tableColumn id="4" xr3:uid="{3B6E882F-295D-45ED-AFA1-B824F78BE80F}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{CDFCC678-2A55-44F4-98F4-A752F86C80D0}" name="price" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{7B967933-54E0-4197-90BA-02740003D24B}" name="rating" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{CDFCC678-2A55-44F4-98F4-A752F86C80D0}" name="price" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{7B967933-54E0-4197-90BA-02740003D24B}" name="rating" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{4085B424-BC45-4516-8F2F-4E61723E45DE}" name="Table11" displayName="Table11" ref="B2:G7" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{4085B424-BC45-4516-8F2F-4E61723E45DE}" name="Table11" displayName="Table11" ref="B2:G7" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="B2:G7" xr:uid="{4085B424-BC45-4516-8F2F-4E61723E45DE}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C60C316F-A75B-4420-9ECC-E7C683652E91}" name="brand"/>
     <tableColumn id="2" xr3:uid="{5D4F5CB5-9DC3-4602-B4DB-1125B37285D0}" name="model"/>
     <tableColumn id="3" xr3:uid="{F1F0F6DE-CE00-4E98-A439-9B55F6E79862}" name="platform"/>
     <tableColumn id="4" xr3:uid="{F98793CD-7209-46DE-930B-B43262054838}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{4D93B0CC-256E-4D8A-BA81-7E3B0F8C15C1}" name="price" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{0DAF1CB5-4E55-463C-8037-08CCB4AC1784}" name="rating" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{4D93B0CC-256E-4D8A-BA81-7E3B0F8C15C1}" name="price" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{0DAF1CB5-4E55-463C-8037-08CCB4AC1784}" name="rating" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{07647B4B-ADAE-49B9-AF20-04A3CBEF2A76}" name="Table14" displayName="Table14" ref="B2:G34" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="14" xr:uid="{07647B4B-ADAE-49B9-AF20-04A3CBEF2A76}" name="Table14" displayName="Table14" ref="B2:G34" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="B2:G34" xr:uid="{07647B4B-ADAE-49B9-AF20-04A3CBEF2A76}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{8B794683-A45B-4580-9EAD-045CF9C202DC}" name="brand"/>
     <tableColumn id="2" xr3:uid="{4BBC79DA-8E64-4567-B20A-B3DF43B32D13}" name="model"/>
     <tableColumn id="3" xr3:uid="{326654EC-E67E-45EB-BD57-E2FE816B68E9}" name="platform"/>
     <tableColumn id="4" xr3:uid="{F42F692D-69A1-47E7-89F9-8ABB126650BA}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{BA2A5026-0272-4166-B014-7F57A6AEFED8}" name="price" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{166B9DDB-9C0D-4B4D-BC05-A43C3EBE75C7}" name="rating" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{BA2A5026-0272-4166-B014-7F57A6AEFED8}" name="price" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{166B9DDB-9C0D-4B4D-BC05-A43C3EBE75C7}" name="rating" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{4C678202-38FD-41AD-90C7-8928EB3E9BF6}" name="Table15" displayName="Table15" ref="B2:G6" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{4C678202-38FD-41AD-90C7-8928EB3E9BF6}" name="Table15" displayName="Table15" ref="B2:G6" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="B2:G6" xr:uid="{4C678202-38FD-41AD-90C7-8928EB3E9BF6}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1E1486B1-02ED-4606-9EA8-7E68501FDDA7}" name="brand"/>
     <tableColumn id="2" xr3:uid="{75ADAE61-FA73-4B93-9A5E-7941AE69FED8}" name="model"/>
     <tableColumn id="3" xr3:uid="{31138AAC-B1AA-47D0-90E7-3B91532B1A05}" name="platform"/>
     <tableColumn id="4" xr3:uid="{BAA01264-E55F-47C4-A256-DC16057D8B7E}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{90C6BEE1-AE7F-4B31-B869-469AAA8A864A}" name="price" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{47918E95-14BB-4227-BB91-8460B27753A2}" name="rating" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{90C6BEE1-AE7F-4B31-B869-469AAA8A864A}" name="price" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{47918E95-14BB-4227-BB91-8460B27753A2}" name="rating" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{906FAACC-6CC3-4061-9964-52F041EEB448}" name="Table2" displayName="Table2" ref="B2:G117" totalsRowShown="0" headerRowDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{906FAACC-6CC3-4061-9964-52F041EEB448}" name="Table2" displayName="Table2" ref="B2:G117" totalsRowShown="0" headerRowDxfId="32">
   <autoFilter ref="B2:G117" xr:uid="{906FAACC-6CC3-4061-9964-52F041EEB448}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{5F8A3743-7B2E-450F-8C88-897EE84D837A}" name="brand"/>
     <tableColumn id="2" xr3:uid="{E9E857EC-966F-4293-8B8A-5A770CB622B7}" name="model"/>
     <tableColumn id="3" xr3:uid="{7F139F35-B4F0-4FA0-B960-045DAD70040D}" name="platform"/>
     <tableColumn id="4" xr3:uid="{721E18BA-7F9E-45A5-8223-92E98854FFC7}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{1D020644-3DBB-439F-9F33-A85C0882378F}" name="price" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{7468242B-F6C3-45B0-B30A-2CC8AF8E0FB5}" name="rating" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{1D020644-3DBB-439F-9F33-A85C0882378F}" name="price" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{7468242B-F6C3-45B0-B30A-2CC8AF8E0FB5}" name="rating" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7D9753A4-423D-4318-A8C3-AB998B29A260}" name="Table3" displayName="Table3" ref="B2:G6" totalsRowShown="0" headerRowDxfId="30">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{7D9753A4-423D-4318-A8C3-AB998B29A260}" name="Table3" displayName="Table3" ref="B2:G6" totalsRowShown="0" headerRowDxfId="29">
   <autoFilter ref="B2:G6" xr:uid="{7D9753A4-423D-4318-A8C3-AB998B29A260}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{C34BC1F2-B54A-4A22-8C98-E780A12D15DB}" name="brand"/>
     <tableColumn id="2" xr3:uid="{84E4E0EC-897E-4B5F-860C-AB13F8108009}" name="model"/>
     <tableColumn id="3" xr3:uid="{29AA954A-8E7B-478D-A771-15D909E50CA7}" name="platform"/>
     <tableColumn id="4" xr3:uid="{32935E93-46CC-46D5-8863-AD1083E94561}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{4D69F091-E8EF-4DDC-AC79-0008684A07BC}" name="price" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{4FD569B8-3944-4D43-A577-12318CBDEAC2}" name="rating" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{4D69F091-E8EF-4DDC-AC79-0008684A07BC}" name="price" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{4FD569B8-3944-4D43-A577-12318CBDEAC2}" name="rating" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0A139ABC-D465-4B40-92B6-8C97957B8ED7}" name="Table4" displayName="Table4" ref="B2:G98" totalsRowShown="0" headerRowDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0A139ABC-D465-4B40-92B6-8C97957B8ED7}" name="Table4" displayName="Table4" ref="B2:G98" totalsRowShown="0" headerRowDxfId="26">
   <autoFilter ref="B2:G98" xr:uid="{0A139ABC-D465-4B40-92B6-8C97957B8ED7}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{F238F6B0-2783-4D23-A079-8FAB1E2EB162}" name="brand"/>
     <tableColumn id="2" xr3:uid="{31BD49F0-A64F-4B64-BC15-2002A9BF9944}" name="model"/>
     <tableColumn id="3" xr3:uid="{C664571D-420E-4D1D-ADCC-A015E3ADB438}" name="platform"/>
     <tableColumn id="4" xr3:uid="{D9FB3E6A-2ACA-4AEB-8831-F5C94D7C8A0A}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{863E17D5-A9C0-4BDC-9F07-9E17EA0FD735}" name="price" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{48D10597-7F5D-4CAC-8FD8-C300DAD12618}" name="rating" dataDxfId="28"/>
+    <tableColumn id="5" xr3:uid="{863E17D5-A9C0-4BDC-9F07-9E17EA0FD735}" name="price" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{48D10597-7F5D-4CAC-8FD8-C300DAD12618}" name="rating" dataDxfId="24"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EE051D89-69F4-42DD-B186-74AB34A74FF2}" name="Table5" displayName="Table5" ref="B2:G17" totalsRowShown="0" headerRowDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EE051D89-69F4-42DD-B186-74AB34A74FF2}" name="Table5" displayName="Table5" ref="B2:G17" totalsRowShown="0" headerRowDxfId="23">
   <autoFilter ref="B2:G17" xr:uid="{EE051D89-69F4-42DD-B186-74AB34A74FF2}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{6377EF2E-C1DF-47E0-B8D4-B1C236445154}" name="brand"/>
     <tableColumn id="2" xr3:uid="{0EAC1C41-D88C-4906-B0FF-492D4DF37727}" name="model"/>
     <tableColumn id="3" xr3:uid="{938BAF50-12CE-4F22-A1E2-4DCA71468076}" name="platform"/>
     <tableColumn id="4" xr3:uid="{5CD7E856-B247-4D29-9B78-4C53F4221A6C}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{1640B708-8860-4D77-ACD6-5DE65B04A3DF}" name="price" dataDxfId="26"/>
-    <tableColumn id="6" xr3:uid="{CC097140-F188-45A3-8526-139F6BEE4C08}" name="rating" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{1640B708-8860-4D77-ACD6-5DE65B04A3DF}" name="price" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{CC097140-F188-45A3-8526-139F6BEE4C08}" name="rating" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2C1BEE2F-536F-4904-BC76-10214916B6E9}" name="Table6" displayName="Table6" ref="B2:G3" totalsRowShown="0" headerRowDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2C1BEE2F-536F-4904-BC76-10214916B6E9}" name="Table6" displayName="Table6" ref="B2:G3" totalsRowShown="0" headerRowDxfId="20">
   <autoFilter ref="B2:G3" xr:uid="{2C1BEE2F-536F-4904-BC76-10214916B6E9}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{47E7C3BE-1277-4151-9943-930751221860}" name="brand"/>
     <tableColumn id="2" xr3:uid="{16CF62A7-45AB-4761-B3D6-FBB953C89456}" name="model"/>
     <tableColumn id="3" xr3:uid="{71205E56-427F-409C-AA48-858ED6DA3893}" name="platform"/>
     <tableColumn id="4" xr3:uid="{69BEFDB9-DB60-4D25-A625-3123F08E7159}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{8C64A8F3-34E9-4549-A9D3-448A40C43A73}" name="price" dataDxfId="23"/>
-    <tableColumn id="6" xr3:uid="{52FD0E9D-0378-4794-9838-54B7BE01E9FE}" name="rating" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{8C64A8F3-34E9-4549-A9D3-448A40C43A73}" name="price" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{52FD0E9D-0378-4794-9838-54B7BE01E9FE}" name="rating" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00DF2E08-75FE-42A6-A78B-7A0356719E91}" name="Table7" displayName="Table7" ref="B2:G28" totalsRowShown="0" headerRowDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00DF2E08-75FE-42A6-A78B-7A0356719E91}" name="Table7" displayName="Table7" ref="B2:G28" totalsRowShown="0" headerRowDxfId="17">
   <autoFilter ref="B2:G28" xr:uid="{00DF2E08-75FE-42A6-A78B-7A0356719E91}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{16864E9E-9C6C-4ADE-9371-CCBD0A603266}" name="brand"/>
     <tableColumn id="2" xr3:uid="{47FAABFD-38B8-4BD2-B6AC-EEBFB844BC2A}" name="model"/>
     <tableColumn id="3" xr3:uid="{C2613F48-F5E2-4737-B86D-3B00728DF669}" name="platform"/>
     <tableColumn id="4" xr3:uid="{16A57B03-E390-4426-A22F-1B6C6D567DC0}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{4DD9B738-E2D7-49DA-9C28-C1016312A6C0}" name="price" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{AE98BD57-7099-42B1-BD96-34598D9C8469}" name="rating" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{4DD9B738-E2D7-49DA-9C28-C1016312A6C0}" name="price" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{AE98BD57-7099-42B1-BD96-34598D9C8469}" name="rating" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{39D7B939-1D12-4E20-89C1-D53803C035F2}" name="Table8" displayName="Table8" ref="B2:G8" totalsRowShown="0" headerRowDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{39D7B939-1D12-4E20-89C1-D53803C035F2}" name="Table8" displayName="Table8" ref="B2:G8" totalsRowShown="0" headerRowDxfId="52">
   <autoFilter ref="B2:G8" xr:uid="{39D7B939-1D12-4E20-89C1-D53803C035F2}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{0585998B-A599-4E85-9C6D-D0A5993AD135}" name="brand"/>
     <tableColumn id="2" xr3:uid="{04A956B8-C210-411F-998F-F5C9BB35471A}" name="model"/>
     <tableColumn id="3" xr3:uid="{07C204C7-3E42-421A-A34F-F48F61D4620D}" name="platform"/>
     <tableColumn id="4" xr3:uid="{E99DAA76-FA52-480C-A231-824B5F140354}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{42E6061D-6621-44D8-85A7-A6CF8AE8F06A}" name="price" dataDxfId="17"/>
-    <tableColumn id="6" xr3:uid="{0562D156-44BF-4498-BB6F-9C9C906DF822}" name="rating" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{42E6061D-6621-44D8-85A7-A6CF8AE8F06A}" name="price" dataDxfId="51"/>
+    <tableColumn id="6" xr3:uid="{0562D156-44BF-4498-BB6F-9C9C906DF822}" name="rating" dataDxfId="50"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{230EFF72-2DCE-4FBC-BFD8-785775B3A380}" name="Table9" displayName="Table9" ref="B2:G5" totalsRowShown="0" headerRowDxfId="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{230EFF72-2DCE-4FBC-BFD8-785775B3A380}" name="Table9" displayName="Table9" ref="B2:G5" totalsRowShown="0" headerRowDxfId="14">
   <autoFilter ref="B2:G5" xr:uid="{230EFF72-2DCE-4FBC-BFD8-785775B3A380}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{BAF19856-4A4D-41E6-BEEE-6BA4B4016F96}" name="brand"/>
     <tableColumn id="2" xr3:uid="{25F52879-9EED-4401-860D-30D1A6F8835D}" name="model"/>
     <tableColumn id="3" xr3:uid="{76B48441-0BB9-4FA0-A118-380DAB019639}" name="platform"/>
     <tableColumn id="4" xr3:uid="{EBE6F2EC-F0F2-4B1D-A94D-A407BD7F5251}" name="product_name"/>
-    <tableColumn id="5" xr3:uid="{5BABA774-C9DC-4BAA-896A-722EDFAA61E2}" name="price" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{CE6E7773-536C-440C-BC12-CF2EF47A6B21}" name="rating" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{5BABA774-C9DC-4BAA-896A-722EDFAA61E2}" name="price" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{CE6E7773-536C-440C-BC12-CF2EF47A6B21}" name="rating" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1444,127 +1458,127 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:24" ht="17.399999999999999">
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="6"/>
+      <c r="X1" s="6"/>
     </row>
     <row r="2" spans="2:24" ht="14.4">
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="4"/>
-      <c r="S2" s="4"/>
-      <c r="T2" s="4"/>
-      <c r="U2" s="4"/>
-      <c r="V2" s="4"/>
-      <c r="W2" s="4"/>
-      <c r="X2" s="4"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+      <c r="X2" s="6"/>
     </row>
     <row r="4" spans="2:24" ht="24.6" customHeight="1">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="F4" s="6" t="s">
+      <c r="E4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="K4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="N4" s="6" t="s">
+      <c r="N4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="O4" s="6" t="s">
+      <c r="O4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="P4" s="6" t="s">
+      <c r="P4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q4" s="6" t="s">
+      <c r="Q4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="R4" s="6" t="s">
+      <c r="R4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="S4" s="6" t="s">
+      <c r="S4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="T4" s="6" t="s">
+      <c r="T4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="U4" s="6" t="s">
+      <c r="U4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="V4" s="6" t="s">
+      <c r="V4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="W4" s="6" t="s">
+      <c r="W4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="X4" s="6" t="s">
+      <c r="X4" s="3" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2402,42 +2416,43 @@
       </c>
     </row>
     <row r="15" spans="2:24">
-      <c r="B15" t="s">
-        <v>5</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="B15" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="G15">
+      <c r="F15" s="8"/>
+      <c r="G15" s="8">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15">
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+      <c r="P15" s="8">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
-      <c r="U15" s="2"/>
-      <c r="V15" s="2"/>
-      <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="10"/>
+      <c r="S15" s="10"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="10"/>
+      <c r="V15" s="10"/>
+      <c r="W15" s="10"/>
+      <c r="X15" s="10"/>
     </row>
     <row r="16" spans="2:24">
       <c r="B16" t="s">
@@ -2701,45 +2716,45 @@
       </c>
     </row>
     <row r="19" spans="2:24">
-      <c r="B19" t="s">
+      <c r="B19" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F19" t="s">
-        <v>43</v>
-      </c>
-      <c r="G19">
+      <c r="F19" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G19" s="8">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19">
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="10"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+      <c r="O19" s="9"/>
+      <c r="P19" s="8">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="2"/>
-      <c r="T19" s="2"/>
-      <c r="U19" s="2"/>
-      <c r="V19" s="2"/>
-      <c r="W19" s="2"/>
-      <c r="X19" s="2"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="10"/>
+      <c r="S19" s="10"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="10"/>
+      <c r="V19" s="10"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="10"/>
     </row>
     <row r="20" spans="2:24">
       <c r="B20" t="s">
@@ -2863,7 +2878,7 @@
         <v>5820.3130808380365</v>
       </c>
       <c r="K21" s="2">
-        <f t="shared" si="2"/>
+        <f>IF(OR(G21&lt;2,H21=0),"",J21/H21*100)</f>
         <v>76.510273677770613</v>
       </c>
       <c r="L21" s="1">
@@ -3632,86 +3647,86 @@
       </c>
     </row>
     <row r="30" spans="2:24">
-      <c r="B30" t="s">
+      <c r="B30" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F30" t="s">
-        <v>42</v>
-      </c>
-      <c r="G30">
+      <c r="F30" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G30" s="8">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="H30" s="1"/>
-      <c r="I30" s="1"/>
-      <c r="J30" s="1"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="1"/>
-      <c r="M30" s="1"/>
-      <c r="N30" s="1"/>
-      <c r="O30" s="1"/>
-      <c r="P30">
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="10"/>
+      <c r="L30" s="9"/>
+      <c r="M30" s="9"/>
+      <c r="N30" s="9"/>
+      <c r="O30" s="9"/>
+      <c r="P30" s="8">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="2"/>
-      <c r="S30" s="2"/>
-      <c r="T30" s="2"/>
-      <c r="U30" s="2"/>
-      <c r="V30" s="2"/>
-      <c r="W30" s="2"/>
-      <c r="X30" s="2"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="10"/>
+      <c r="S30" s="10"/>
+      <c r="T30" s="10"/>
+      <c r="U30" s="10"/>
+      <c r="V30" s="10"/>
+      <c r="W30" s="10"/>
+      <c r="X30" s="10"/>
     </row>
     <row r="31" spans="2:24">
-      <c r="B31" t="s">
+      <c r="B31" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E31" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="F31" t="s">
-        <v>43</v>
-      </c>
-      <c r="G31">
+      <c r="F31" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G31" s="8">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="1"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="1"/>
-      <c r="M31" s="1"/>
-      <c r="N31" s="1"/>
-      <c r="O31" s="1"/>
-      <c r="P31">
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="10"/>
+      <c r="L31" s="9"/>
+      <c r="M31" s="9"/>
+      <c r="N31" s="9"/>
+      <c r="O31" s="9"/>
+      <c r="P31" s="8">
         <f>0</f>
         <v>0</v>
       </c>
-      <c r="Q31" s="2"/>
-      <c r="R31" s="2"/>
-      <c r="S31" s="2"/>
-      <c r="T31" s="2"/>
-      <c r="U31" s="2"/>
-      <c r="V31" s="2"/>
-      <c r="W31" s="2"/>
-      <c r="X31" s="2"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="10"/>
+      <c r="S31" s="10"/>
+      <c r="T31" s="10"/>
+      <c r="U31" s="10"/>
+      <c r="V31" s="10"/>
+      <c r="W31" s="10"/>
+      <c r="X31" s="10"/>
     </row>
     <row r="32" spans="2:24">
       <c r="B32" t="s">
@@ -4094,22 +4109,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -4866,22 +4881,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -5004,22 +5019,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="4" t="s">
         <v>49</v>
       </c>
     </row>
@@ -5041,22 +5056,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -5697,22 +5712,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -5813,22 +5828,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="38.4" customHeight="1">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -8027,22 +8042,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -8147,22 +8162,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -10035,22 +10050,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -10363,22 +10378,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -10423,22 +10438,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -10963,22 +10978,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -11117,22 +11132,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:7">
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>